<commit_message>
Mise à jour de la feuille de route et du modèle financier
Page de garde avec le logo, retrait de la partie financement personnel,
abandon de l'onduleur UPS (kit 316 000 CFA, réserve 294 000 CFA),
rédaction retravaillée.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138tNhYaE2Tp89oR11QdC4C
</commit_message>
<xml_diff>
--- a/ScentSenegal_Modele_Financier.xlsx
+++ b/ScentSenegal_Modele_Financier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hypothèses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Économie unitaire" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Projection 24 mois" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothèses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Économie unitaire" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projection 24 mois" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D37"/>
+  <dimension ref="B1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1084,7 +1084,7 @@
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Diffuseur A300 (compact)</t>
+          <t>Diffuseur SS100 (compact)</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
@@ -1099,7 +1099,7 @@
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Diffuseur X2000 (grand format)</t>
+          <t>Diffuseur SS200 (grand format)</t>
         </is>
       </c>
       <c r="C24" s="12" t="n">
@@ -1110,150 +1110,135 @@
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Onduleur UPS</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>35000</v>
+          <t>Taux de douane / import sur le matériel</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0.2</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Anti-coupures</t>
+          <t>Estimation — À VÉRIFIER</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Taux de douane / import sur le matériel</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Estimation — À VÉRIFIER</t>
-        </is>
-      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Trésorerie &amp; financement</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Trésorerie &amp; financement</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Capital business d'ouverture</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>610000</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>≈ 1000 $ au lancement (mois 4 du plan)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Capital business d'ouverture</t>
+          <t>Apport personnel / mois</t>
         </is>
       </c>
       <c r="C28" s="12" t="n">
-        <v>610000</v>
+        <v>305000</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>≈ 1000 $ au lancement (mois 4 du plan)</t>
+          <t>≈ 500 $/mois (règle des 50%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Apport personnel / mois</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="n">
-        <v>305000</v>
+          <t>Dernier mois d'apport personnel</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>9</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>≈ 500 $/mois (règle des 50%)</t>
+          <t>Au-delà : business autofinancé</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Dernier mois d'apport personnel</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="n">
-        <v>9</v>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Au-delà : business autofinancé</t>
-        </is>
-      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Essai gratuit</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Essai gratuit</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Décalage de revenu</t>
         </is>
       </c>
-      <c r="C32" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="C31" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Mois d'essai gratuit : le client paie le mois SUIVANT son installation</t>
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>CapEx matériel par client (calculé, avec douane)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr"/>
+    </row>
     <row r="34">
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>CapEx matériel par client (calculé, avec douane)</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Découverte (1× SS100)</t>
+        </is>
+      </c>
+      <c r="C34" s="16">
+        <f>(Hypothèses!$C$23)*(1+Hypothèses!$C$25)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Découverte (1× A300)</t>
+          <t>Confort (2× SS100)</t>
         </is>
       </c>
       <c r="C35" s="16">
-        <f>(Hypothèses!$C$23)*(1+Hypothèses!$C$26)</f>
+        <f>(2*Hypothèses!$C$23)*(1+Hypothèses!$C$25)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Confort (2× A300)</t>
+          <t>Prestige (1× SS200 + 2× SS100)</t>
         </is>
       </c>
       <c r="C36" s="16">
-        <f>(2*Hypothèses!$C$23)*(1+Hypothèses!$C$26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Prestige (1× X2000 + 2× A300 + UPS)</t>
-        </is>
-      </c>
-      <c r="C37" s="16">
-        <f>(Hypothèses!$C$24+2*Hypothèses!$C$23+Hypothèses!$C$25)*(1+Hypothèses!$C$26)</f>
+        <f>(Hypothèses!$C$24+2*Hypothèses!$C$23)*(1+Hypothèses!$C$25)</f>
         <v/>
       </c>
     </row>
@@ -1450,15 +1435,15 @@
         </is>
       </c>
       <c r="C12" s="18">
+        <f>Hypothèses!$C$34</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
         <f>Hypothèses!$C$35</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="E12" s="18">
         <f>Hypothèses!$C$36</f>
-        <v/>
-      </c>
-      <c r="E12" s="18">
-        <f>Hypothèses!$C$37</f>
         <v/>
       </c>
     </row>
@@ -3027,99 +3012,99 @@
         </is>
       </c>
       <c r="B17" s="18">
-        <f>-(B3*Hypothèses!$C$35+B4*Hypothèses!$C$36+B5*Hypothèses!$C$37)</f>
+        <f>-(B3*Hypothèses!$C$34+B4*Hypothèses!$C$35+B5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="C17" s="18">
-        <f>-(C3*Hypothèses!$C$35+C4*Hypothèses!$C$36+C5*Hypothèses!$C$37)</f>
+        <f>-(C3*Hypothèses!$C$34+C4*Hypothèses!$C$35+C5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="D17" s="18">
-        <f>-(D3*Hypothèses!$C$35+D4*Hypothèses!$C$36+D5*Hypothèses!$C$37)</f>
+        <f>-(D3*Hypothèses!$C$34+D4*Hypothèses!$C$35+D5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="E17" s="18">
-        <f>-(E3*Hypothèses!$C$35+E4*Hypothèses!$C$36+E5*Hypothèses!$C$37)</f>
+        <f>-(E3*Hypothèses!$C$34+E4*Hypothèses!$C$35+E5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="F17" s="18">
-        <f>-(F3*Hypothèses!$C$35+F4*Hypothèses!$C$36+F5*Hypothèses!$C$37)</f>
+        <f>-(F3*Hypothèses!$C$34+F4*Hypothèses!$C$35+F5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="G17" s="18">
-        <f>-(G3*Hypothèses!$C$35+G4*Hypothèses!$C$36+G5*Hypothèses!$C$37)</f>
+        <f>-(G3*Hypothèses!$C$34+G4*Hypothèses!$C$35+G5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="H17" s="18">
-        <f>-(H3*Hypothèses!$C$35+H4*Hypothèses!$C$36+H5*Hypothèses!$C$37)</f>
+        <f>-(H3*Hypothèses!$C$34+H4*Hypothèses!$C$35+H5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="I17" s="18">
-        <f>-(I3*Hypothèses!$C$35+I4*Hypothèses!$C$36+I5*Hypothèses!$C$37)</f>
+        <f>-(I3*Hypothèses!$C$34+I4*Hypothèses!$C$35+I5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="J17" s="18">
-        <f>-(J3*Hypothèses!$C$35+J4*Hypothèses!$C$36+J5*Hypothèses!$C$37)</f>
+        <f>-(J3*Hypothèses!$C$34+J4*Hypothèses!$C$35+J5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>-(K3*Hypothèses!$C$35+K4*Hypothèses!$C$36+K5*Hypothèses!$C$37)</f>
+        <f>-(K3*Hypothèses!$C$34+K4*Hypothèses!$C$35+K5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>-(L3*Hypothèses!$C$35+L4*Hypothèses!$C$36+L5*Hypothèses!$C$37)</f>
+        <f>-(L3*Hypothèses!$C$34+L4*Hypothèses!$C$35+L5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="M17" s="18">
-        <f>-(M3*Hypothèses!$C$35+M4*Hypothèses!$C$36+M5*Hypothèses!$C$37)</f>
+        <f>-(M3*Hypothèses!$C$34+M4*Hypothèses!$C$35+M5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="N17" s="18">
-        <f>-(N3*Hypothèses!$C$35+N4*Hypothèses!$C$36+N5*Hypothèses!$C$37)</f>
+        <f>-(N3*Hypothèses!$C$34+N4*Hypothèses!$C$35+N5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="O17" s="18">
-        <f>-(O3*Hypothèses!$C$35+O4*Hypothèses!$C$36+O5*Hypothèses!$C$37)</f>
+        <f>-(O3*Hypothèses!$C$34+O4*Hypothèses!$C$35+O5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="P17" s="18">
-        <f>-(P3*Hypothèses!$C$35+P4*Hypothèses!$C$36+P5*Hypothèses!$C$37)</f>
+        <f>-(P3*Hypothèses!$C$34+P4*Hypothèses!$C$35+P5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="Q17" s="18">
-        <f>-(Q3*Hypothèses!$C$35+Q4*Hypothèses!$C$36+Q5*Hypothèses!$C$37)</f>
+        <f>-(Q3*Hypothèses!$C$34+Q4*Hypothèses!$C$35+Q5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="R17" s="18">
-        <f>-(R3*Hypothèses!$C$35+R4*Hypothèses!$C$36+R5*Hypothèses!$C$37)</f>
+        <f>-(R3*Hypothèses!$C$34+R4*Hypothèses!$C$35+R5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="S17" s="18">
-        <f>-(S3*Hypothèses!$C$35+S4*Hypothèses!$C$36+S5*Hypothèses!$C$37)</f>
+        <f>-(S3*Hypothèses!$C$34+S4*Hypothèses!$C$35+S5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="T17" s="18">
-        <f>-(T3*Hypothèses!$C$35+T4*Hypothèses!$C$36+T5*Hypothèses!$C$37)</f>
+        <f>-(T3*Hypothèses!$C$34+T4*Hypothèses!$C$35+T5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="U17" s="18">
-        <f>-(U3*Hypothèses!$C$35+U4*Hypothèses!$C$36+U5*Hypothèses!$C$37)</f>
+        <f>-(U3*Hypothèses!$C$34+U4*Hypothèses!$C$35+U5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="V17" s="18">
-        <f>-(V3*Hypothèses!$C$35+V4*Hypothèses!$C$36+V5*Hypothèses!$C$37)</f>
+        <f>-(V3*Hypothèses!$C$34+V4*Hypothèses!$C$35+V5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="W17" s="18">
-        <f>-(W3*Hypothèses!$C$35+W4*Hypothèses!$C$36+W5*Hypothèses!$C$37)</f>
+        <f>-(W3*Hypothèses!$C$34+W4*Hypothèses!$C$35+W5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="X17" s="18">
-        <f>-(X3*Hypothèses!$C$35+X4*Hypothèses!$C$36+X5*Hypothèses!$C$37)</f>
+        <f>-(X3*Hypothèses!$C$34+X4*Hypothèses!$C$35+X5*Hypothèses!$C$36)</f>
         <v/>
       </c>
       <c r="Y17" s="18">
-        <f>-(Y3*Hypothèses!$C$35+Y4*Hypothèses!$C$36+Y5*Hypothèses!$C$37)</f>
+        <f>-(Y3*Hypothèses!$C$34+Y4*Hypothèses!$C$35+Y5*Hypothèses!$C$36)</f>
         <v/>
       </c>
     </row>
@@ -3130,99 +3115,99 @@
         </is>
       </c>
       <c r="B18" s="18">
-        <f>IF(B2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(B2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="C18" s="18">
-        <f>IF(C2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(C2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="D18" s="18">
-        <f>IF(D2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(D2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="E18" s="18">
-        <f>IF(E2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(E2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="F18" s="18">
-        <f>IF(F2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(F2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="G18" s="18">
-        <f>IF(G2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(G2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="H18" s="18">
-        <f>IF(H2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(H2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="I18" s="18">
-        <f>IF(I2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(I2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="J18" s="18">
-        <f>IF(J2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(J2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="K18" s="18">
-        <f>IF(K2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(K2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="L18" s="18">
-        <f>IF(L2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(L2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="M18" s="18">
-        <f>IF(M2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(M2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="N18" s="18">
-        <f>IF(N2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(N2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="O18" s="18">
-        <f>IF(O2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(O2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="P18" s="18">
-        <f>IF(P2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(P2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="Q18" s="18">
-        <f>IF(Q2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(Q2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="R18" s="18">
-        <f>IF(R2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(R2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="S18" s="18">
-        <f>IF(S2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(S2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="T18" s="18">
-        <f>IF(T2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(T2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="U18" s="18">
-        <f>IF(U2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(U2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="V18" s="18">
-        <f>IF(V2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(V2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="W18" s="18">
-        <f>IF(W2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(W2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="X18" s="18">
-        <f>IF(X2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(X2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
       <c r="Y18" s="18">
-        <f>IF(Y2&lt;=Hypothèses!$C$30,Hypothèses!$C$29,0)</f>
+        <f>IF(Y2&lt;=Hypothèses!$C$29,Hypothèses!$C$28,0)</f>
         <v/>
       </c>
     </row>
@@ -3335,7 +3320,7 @@
         </is>
       </c>
       <c r="B20" s="6">
-        <f>Hypothèses!$C$28+B19</f>
+        <f>Hypothèses!$C$27+B19</f>
         <v/>
       </c>
       <c r="C20" s="6">

</xml_diff>